<commit_message>
cycle 2026-09-14 18:16 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I498"/>
+  <dimension ref="A1:I504"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19497,6 +19497,232 @@
       <c r="I498" s="4" t="inlineStr">
         <is>
           <t>BAC's 10-hour average price ($62.64) is above its 30-hour average ($62.63). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="499" ht="40" customHeight="1">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B499" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F499" s="2" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="G499" s="2" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="H499" s="2" t="inlineStr"/>
+      <c r="I499" s="4" t="inlineStr">
+        <is>
+          <t>NFLX is ranked #1 out of 25 stocks by momentum. It gained 5.05% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="500" ht="40" customHeight="1">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C500" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E500" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F500" s="2" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="G500" s="2" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="H500" s="2" t="inlineStr"/>
+      <c r="I500" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #2 out of 25 stocks by momentum. It gained 3.10% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="501" ht="40" customHeight="1">
+      <c r="A501" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B501" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C501" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D501" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E501" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F501" s="8" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="G501" s="8" t="n">
+        <v>109.44</v>
+      </c>
+      <c r="H501" s="12" t="n">
+        <v>3.54</v>
+      </c>
+      <c r="I501" s="11" t="inlineStr">
+        <is>
+          <t>WMT's RSI climbed to 87.9, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="502" ht="40" customHeight="1">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B502" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C502" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E502" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F502" s="2" t="n">
+        <v>59.33</v>
+      </c>
+      <c r="G502" s="2" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="H502" s="2" t="inlineStr"/>
+      <c r="I502" s="4" t="inlineStr">
+        <is>
+          <t>BAC's RSI is 16.4, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="503" ht="40" customHeight="1">
+      <c r="A503" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B503" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C503" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D503" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E503" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F503" s="8" t="n">
+        <v>59.33</v>
+      </c>
+      <c r="G503" s="8" t="n">
+        <v>118.67</v>
+      </c>
+      <c r="H503" s="10" t="n">
+        <v>-7.08</v>
+      </c>
+      <c r="I503" s="11" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average ($61.96) dropped below its 30-hour average ($62.38). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="504" ht="40" customHeight="1">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-14 18:16</t>
+        </is>
+      </c>
+      <c r="B504" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C504" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E504" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F504" s="2" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="G504" s="2" t="n">
+        <v>80.63</v>
+      </c>
+      <c r="H504" s="2" t="inlineStr"/>
+      <c r="I504" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average price ($78.80) is above its 30-hour average ($77.14). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -19565,7 +19791,7 @@
         <v>628.88</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>628.88</v>
+        <v>438.81</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -19584,19 +19810,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>660.87</v>
+        <v>664.4</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>265.21</v>
+        <v>255.98</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>60.87</v>
+        <v>64.40000000000001</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>10.14</v>
+        <v>10.73</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -19606,19 +19832,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>585.61</v>
+        <v>578.53</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>264.45</v>
+        <v>302.49</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-14.39</v>
+        <v>-21.47</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-2.4</v>
+        <v>-3.58</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -19658,7 +19884,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-11 22:16 UTC</t>
+          <t>Generated: 2026-09-14 18:16 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-15 17:24 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I504"/>
+  <dimension ref="A1:I509"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19723,6 +19723,197 @@
       <c r="I504" s="4" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average price ($78.80) is above its 30-hour average ($77.14). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="505" ht="40" customHeight="1">
+      <c r="A505" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:24</t>
+        </is>
+      </c>
+      <c r="B505" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C505" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D505" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E505" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F505" s="8" t="n">
+        <v>78.31</v>
+      </c>
+      <c r="G505" s="8" t="n">
+        <v>78.31</v>
+      </c>
+      <c r="H505" s="10" t="n">
+        <v>-2.32</v>
+      </c>
+      <c r="I505" s="11" t="inlineStr">
+        <is>
+          <t>NFLX lost momentum: down 1.89% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="506" ht="40" customHeight="1">
+      <c r="A506" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:24</t>
+        </is>
+      </c>
+      <c r="B506" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C506" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D506" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E506" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F506" s="8" t="n">
+        <v>108.61</v>
+      </c>
+      <c r="G506" s="8" t="n">
+        <v>108.61</v>
+      </c>
+      <c r="H506" s="10" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="I506" s="11" t="inlineStr">
+        <is>
+          <t>WMT lost momentum: down 0.46% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="507" ht="40" customHeight="1">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:24</t>
+        </is>
+      </c>
+      <c r="B507" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="E507" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F507" s="2" t="n">
+        <v>146.8</v>
+      </c>
+      <c r="G507" s="2" t="n">
+        <v>146.8</v>
+      </c>
+      <c r="H507" s="2" t="inlineStr"/>
+      <c r="I507" s="4" t="inlineStr">
+        <is>
+          <t>PG's 10-hour average price ($146.36) is above its 30-hour average ($144.56). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="508" ht="40" customHeight="1">
+      <c r="A508" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:24</t>
+        </is>
+      </c>
+      <c r="B508" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C508" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D508" s="8" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="E508" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F508" s="8" t="n">
+        <v>86.20999999999999</v>
+      </c>
+      <c r="G508" s="8" t="n">
+        <v>86.20999999999999</v>
+      </c>
+      <c r="H508" s="10" t="n">
+        <v>-7.78</v>
+      </c>
+      <c r="I508" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: SO dropped 8.3% from the entry price (bought at $93.99, now $86.21). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="509" ht="40" customHeight="1">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-15 17:24</t>
+        </is>
+      </c>
+      <c r="B509" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="F509" s="2" t="n">
+        <v>26.85</v>
+      </c>
+      <c r="G509" s="2" t="n">
+        <v>107.42</v>
+      </c>
+      <c r="H509" s="2" t="inlineStr"/>
+      <c r="I509" s="4" t="inlineStr">
+        <is>
+          <t>T pays a 4.19% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($26.85) is above its 30-hour average ($25.97), confirming a healthy trend. Buying to collect steady income while holding.</t>
         </is>
       </c>
     </row>
@@ -19788,19 +19979,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>628.88</v>
+        <v>625.73</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>438.81</v>
+        <v>625.73</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>28.88</v>
+        <v>25.73</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.81</v>
+        <v>4.29</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -19835,7 +20026,7 @@
         <v>578.53</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>302.49</v>
+        <v>155.69</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -19854,19 +20045,19 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>569.95</v>
+        <v>562.17</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>23.26</v>
+        <v>2.05</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-30.05</v>
+        <v>-37.83</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-5.01</v>
+        <v>-6.3</v>
       </c>
     </row>
     <row r="6">
@@ -19884,7 +20075,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-14 22:57 UTC</t>
+          <t>Generated: 2026-09-15 17:24 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-16 17:23 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I509"/>
+  <dimension ref="A1:I512"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -19914,6 +19914,121 @@
       <c r="I509" s="4" t="inlineStr">
         <is>
           <t>T pays a 4.19% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($26.85) is above its 30-hour average ($25.97), confirming a healthy trend. Buying to collect steady income while holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="510" ht="40" customHeight="1">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-16 17:23</t>
+        </is>
+      </c>
+      <c r="B510" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C510" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E510" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F510" s="2" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="G510" s="2" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="H510" s="2" t="inlineStr"/>
+      <c r="I510" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's RSI is 17.6, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="511" ht="40" customHeight="1">
+      <c r="A511" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-16 17:23</t>
+        </is>
+      </c>
+      <c r="B511" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C511" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D511" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E511" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F511" s="8" t="n">
+        <v>88.45</v>
+      </c>
+      <c r="G511" s="8" t="n">
+        <v>88.45</v>
+      </c>
+      <c r="H511" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I511" s="11" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average ($88.49) dropped below its 30-hour average ($88.54). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="512" ht="40" customHeight="1">
+      <c r="A512" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-16 17:23</t>
+        </is>
+      </c>
+      <c r="B512" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C512" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D512" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E512" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F512" s="8" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="G512" s="8" t="n">
+        <v>77.26000000000001</v>
+      </c>
+      <c r="H512" s="10" t="n">
+        <v>-3.36</v>
+      </c>
+      <c r="I512" s="11" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average ($77.78) dropped below its 30-hour average ($77.91). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -20004,7 +20119,7 @@
         <v>664.4</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>255.98</v>
+        <v>178.71</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
@@ -20023,19 +20138,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>578.53</v>
+        <v>575.27</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>155.69</v>
+        <v>321.4</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-21.47</v>
+        <v>-24.73</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-3.58</v>
+        <v>-4.12</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -20075,7 +20190,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-15 22:43 UTC</t>
+          <t>Generated: 2026-09-16 17:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-17 17:22 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I512"/>
+  <dimension ref="A1:I517"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20029,6 +20029,197 @@
       <c r="I512" s="11" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average ($77.78) dropped below its 30-hour average ($77.91). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="513" ht="40" customHeight="1">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:22</t>
+        </is>
+      </c>
+      <c r="B513" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C513" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E513" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F513" s="2" t="n">
+        <v>106.74</v>
+      </c>
+      <c r="G513" s="2" t="n">
+        <v>106.74</v>
+      </c>
+      <c r="H513" s="2" t="inlineStr"/>
+      <c r="I513" s="4" t="inlineStr">
+        <is>
+          <t>WMT's RSI is 29.0, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="514" ht="40" customHeight="1">
+      <c r="A514" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:22</t>
+        </is>
+      </c>
+      <c r="B514" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C514" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D514" s="8" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="E514" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F514" s="8" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="G514" s="8" t="n">
+        <v>146.66</v>
+      </c>
+      <c r="H514" s="10" t="n">
+        <v>-1.08</v>
+      </c>
+      <c r="I514" s="11" t="inlineStr">
+        <is>
+          <t>MRK's RSI climbed to 78.2, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="515" ht="40" customHeight="1">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:22</t>
+        </is>
+      </c>
+      <c r="B515" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C515" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="E515" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F515" s="2" t="n">
+        <v>211.04</v>
+      </c>
+      <c r="G515" s="2" t="n">
+        <v>211.04</v>
+      </c>
+      <c r="H515" s="2" t="inlineStr"/>
+      <c r="I515" s="4" t="inlineStr">
+        <is>
+          <t>CVX's RSI is 29.4, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="516" ht="40" customHeight="1">
+      <c r="A516" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:22</t>
+        </is>
+      </c>
+      <c r="B516" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C516" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D516" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E516" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F516" s="8" t="n">
+        <v>106.74</v>
+      </c>
+      <c r="G516" s="8" t="n">
+        <v>106.74</v>
+      </c>
+      <c r="H516" s="10" t="n">
+        <v>-0.33</v>
+      </c>
+      <c r="I516" s="11" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average ($107.51) dropped below its 30-hour average ($108.07). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="517" ht="40" customHeight="1">
+      <c r="A517" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-17 17:22</t>
+        </is>
+      </c>
+      <c r="B517" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C517" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D517" s="8" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E517" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F517" s="8" t="n">
+        <v>57.19</v>
+      </c>
+      <c r="G517" s="8" t="n">
+        <v>57.19</v>
+      </c>
+      <c r="H517" s="10" t="n">
+        <v>-5.33</v>
+      </c>
+      <c r="I517" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: O dropped 8.5% from the entry price (bought at $62.51, now $57.19). Selling automatically to protect capital before losses grow further.</t>
         </is>
       </c>
     </row>
@@ -20116,19 +20307,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>664.4</v>
+        <v>663.3200000000001</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>178.71</v>
+        <v>7.6</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>64.40000000000001</v>
+        <v>63.32</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>10.73</v>
+        <v>10.55</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -20138,19 +20329,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>575.27</v>
+        <v>574.9400000000001</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>321.4</v>
+        <v>428.14</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-24.73</v>
+        <v>-25.06</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.12</v>
+        <v>-4.18</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -20160,19 +20351,19 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>562.17</v>
+        <v>556.84</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>2.05</v>
+        <v>59.23</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-37.83</v>
+        <v>-43.16</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-6.3</v>
+        <v>-7.19</v>
       </c>
     </row>
     <row r="6">
@@ -20190,7 +20381,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-16 22:39 UTC</t>
+          <t>Generated: 2026-09-17 17:22 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-18 16:50 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I517"/>
+  <dimension ref="A1:I520"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20220,6 +20220,121 @@
       <c r="I517" s="11" t="inlineStr">
         <is>
           <t>STOP-LOSS: O dropped 8.5% from the entry price (bought at $62.51, now $57.19). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="518" ht="40" customHeight="1">
+      <c r="A518" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:50</t>
+        </is>
+      </c>
+      <c r="B518" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C518" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D518" s="8" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E518" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F518" s="8" t="n">
+        <v>130.26</v>
+      </c>
+      <c r="G518" s="8" t="n">
+        <v>130.26</v>
+      </c>
+      <c r="H518" s="10" t="n">
+        <v>-11.75</v>
+      </c>
+      <c r="I518" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: PEP dropped 8.3% from the entry price (bought at $142.01, now $130.26). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="519" ht="40" customHeight="1">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:50</t>
+        </is>
+      </c>
+      <c r="B519" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C519" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E519" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F519" s="2" t="n">
+        <v>130.26</v>
+      </c>
+      <c r="G519" s="2" t="n">
+        <v>130.26</v>
+      </c>
+      <c r="H519" s="2" t="inlineStr"/>
+      <c r="I519" s="4" t="inlineStr">
+        <is>
+          <t>PEP's RSI is 17.6, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="520" ht="40" customHeight="1">
+      <c r="A520" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-18 16:50</t>
+        </is>
+      </c>
+      <c r="B520" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C520" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D520" s="8" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="E520" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F520" s="8" t="n">
+        <v>146.29</v>
+      </c>
+      <c r="G520" s="8" t="n">
+        <v>146.29</v>
+      </c>
+      <c r="H520" s="10" t="n">
+        <v>-0.51</v>
+      </c>
+      <c r="I520" s="11" t="inlineStr">
+        <is>
+          <t>PG's 10-hour average ($146.83) dropped below its 30-hour average ($146.88). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -20307,7 +20422,7 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>663.3200000000001</v>
+        <v>651.5700000000001</v>
       </c>
       <c r="C3" s="16" t="n">
         <v>7.6</v>
@@ -20316,10 +20431,10 @@
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>63.32</v>
+        <v>51.57</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>10.55</v>
+        <v>8.59</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -20329,19 +20444,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>574.9400000000001</v>
+        <v>574.4299999999999</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>428.14</v>
+        <v>574.4299999999999</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-25.06</v>
+        <v>-25.57</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.18</v>
+        <v>-4.26</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -20381,7 +20496,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-17 22:41 UTC</t>
+          <t>Generated: 2026-09-18 16:50 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-18 19:14 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I520"/>
+  <dimension ref="A1:I521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20335,6 +20335,43 @@
       <c r="I520" s="11" t="inlineStr">
         <is>
           <t>PG's 10-hour average ($146.83) dropped below its 30-hour average ($146.88). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="521" ht="40" customHeight="1">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-18 19:14</t>
+        </is>
+      </c>
+      <c r="B521" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C521" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E521" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F521" s="2" t="n">
+        <v>107.54</v>
+      </c>
+      <c r="G521" s="2" t="n">
+        <v>107.54</v>
+      </c>
+      <c r="H521" s="2" t="inlineStr"/>
+      <c r="I521" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 0.90% over the last 10 hours, showing strong upward price pressure.</t>
         </is>
       </c>
     </row>
@@ -20403,7 +20440,7 @@
         <v>625.73</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>625.73</v>
+        <v>518.1799999999999</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -20496,7 +20533,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-18 16:50 UTC</t>
+          <t>Generated: 2026-09-18 19:14 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-21 18:23 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I521"/>
+  <dimension ref="A1:I522"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20372,6 +20372,45 @@
       <c r="I521" s="4" t="inlineStr">
         <is>
           <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 0.90% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="522" ht="40" customHeight="1">
+      <c r="A522" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-21 18:23</t>
+        </is>
+      </c>
+      <c r="B522" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C522" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D522" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E522" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F522" s="8" t="n">
+        <v>107.51</v>
+      </c>
+      <c r="G522" s="8" t="n">
+        <v>107.51</v>
+      </c>
+      <c r="H522" s="10" t="n">
+        <v>-0.03</v>
+      </c>
+      <c r="I522" s="11" t="inlineStr">
+        <is>
+          <t>WMT dropped out of the top 5 momentum stocks (current momentum: 0.30%). Rotating into stronger performers.</t>
         </is>
       </c>
     </row>
@@ -20437,19 +20476,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>625.73</v>
+        <v>625.6900000000001</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>518.1799999999999</v>
+        <v>625.6900000000001</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>25.73</v>
+        <v>25.69</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.29</v>
+        <v>4.28</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -20533,7 +20572,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-18 22:19 UTC</t>
+          <t>Generated: 2026-09-21 18:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-22 17:26 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I522"/>
+  <dimension ref="A1:I525"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20411,6 +20411,119 @@
       <c r="I522" s="11" t="inlineStr">
         <is>
           <t>WMT dropped out of the top 5 momentum stocks (current momentum: 0.30%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="523" ht="40" customHeight="1">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 17:26</t>
+        </is>
+      </c>
+      <c r="B523" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C523" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E523" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F523" s="2" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="G523" s="2" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="H523" s="2" t="inlineStr"/>
+      <c r="I523" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #4 out of 25 stocks by momentum. It gained 2.44% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="524" ht="40" customHeight="1">
+      <c r="A524" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-22 17:26</t>
+        </is>
+      </c>
+      <c r="B524" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C524" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D524" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E524" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F524" s="8" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="G524" s="8" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="H524" s="12" t="n">
+        <v>3.14</v>
+      </c>
+      <c r="I524" s="11" t="inlineStr">
+        <is>
+          <t>WMT's RSI climbed to 78.2, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="525" ht="40" customHeight="1">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-22 17:26</t>
+        </is>
+      </c>
+      <c r="B525" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C525" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E525" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F525" s="2" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="G525" s="2" t="n">
+        <v>109.87</v>
+      </c>
+      <c r="H525" s="2" t="inlineStr"/>
+      <c r="I525" s="4" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average price ($108.09) is above its 30-hour average ($107.52). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -20479,7 +20592,7 @@
         <v>625.6900000000001</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>625.6900000000001</v>
+        <v>515.8200000000001</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -20498,19 +20611,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>651.5700000000001</v>
+        <v>654.7</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>7.6</v>
+        <v>117.47</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>51.57</v>
+        <v>54.7</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>8.59</v>
+        <v>9.119999999999999</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -20523,7 +20636,7 @@
         <v>574.4299999999999</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>574.4299999999999</v>
+        <v>464.56</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -20572,7 +20685,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-21 23:00 UTC</t>
+          <t>Generated: 2026-09-22 17:26 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-23 17:36 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I525"/>
+  <dimension ref="A1:I526"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20524,6 +20524,43 @@
       <c r="I525" s="4" t="inlineStr">
         <is>
           <t>WMT's 10-hour average price ($108.09) is above its 30-hour average ($107.52). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="526" ht="40" customHeight="1">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-23 17:36</t>
+        </is>
+      </c>
+      <c r="B526" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C526" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E526" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F526" s="2" t="n">
+        <v>87.94</v>
+      </c>
+      <c r="G526" s="2" t="n">
+        <v>87.94</v>
+      </c>
+      <c r="H526" s="2" t="inlineStr"/>
+      <c r="I526" s="4" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average price ($88.35) is above its 30-hour average ($88.06). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -20636,7 +20673,7 @@
         <v>574.4299999999999</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>464.56</v>
+        <v>376.62</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -20685,7 +20722,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-22 22:44 UTC</t>
+          <t>Generated: 2026-09-23 17:36 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-24 17:39 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I526"/>
+  <dimension ref="A1:I527"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20561,6 +20561,45 @@
       <c r="I526" s="4" t="inlineStr">
         <is>
           <t>KO's 10-hour average price ($88.35) is above its 30-hour average ($88.06). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="527" ht="40" customHeight="1">
+      <c r="A527" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-24 17:39</t>
+        </is>
+      </c>
+      <c r="B527" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C527" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D527" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E527" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F527" s="8" t="n">
+        <v>108.35</v>
+      </c>
+      <c r="G527" s="8" t="n">
+        <v>108.35</v>
+      </c>
+      <c r="H527" s="10" t="n">
+        <v>-1.52</v>
+      </c>
+      <c r="I527" s="11" t="inlineStr">
+        <is>
+          <t>WMT lost momentum: down 1.33% over the last 10 hours. Selling to avoid further losses.</t>
         </is>
       </c>
     </row>
@@ -20626,19 +20665,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>625.6900000000001</v>
+        <v>624.17</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>515.8200000000001</v>
+        <v>624.17</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>25.69</v>
+        <v>24.17</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.28</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -20722,7 +20761,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-23 22:41 UTC</t>
+          <t>Generated: 2026-09-24 17:39 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-25 17:39 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I527"/>
+  <dimension ref="A1:I530"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20600,6 +20600,121 @@
       <c r="I527" s="11" t="inlineStr">
         <is>
           <t>WMT lost momentum: down 1.33% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="528" ht="40" customHeight="1">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-25 17:39</t>
+        </is>
+      </c>
+      <c r="B528" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C528" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E528" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F528" s="2" t="n">
+        <v>107.82</v>
+      </c>
+      <c r="G528" s="2" t="n">
+        <v>107.82</v>
+      </c>
+      <c r="H528" s="2" t="inlineStr"/>
+      <c r="I528" s="4" t="inlineStr">
+        <is>
+          <t>WMT's RSI is 25.1, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="529" ht="40" customHeight="1">
+      <c r="A529" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-25 17:39</t>
+        </is>
+      </c>
+      <c r="B529" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C529" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D529" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E529" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F529" s="8" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="G529" s="8" t="n">
+        <v>112.99</v>
+      </c>
+      <c r="H529" s="10" t="n">
+        <v>-5.68</v>
+      </c>
+      <c r="I529" s="11" t="inlineStr">
+        <is>
+          <t>BAC's RSI climbed to 66.4, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="530" ht="40" customHeight="1">
+      <c r="A530" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-25 17:39</t>
+        </is>
+      </c>
+      <c r="B530" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C530" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D530" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E530" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F530" s="8" t="n">
+        <v>107.82</v>
+      </c>
+      <c r="G530" s="8" t="n">
+        <v>107.82</v>
+      </c>
+      <c r="H530" s="10" t="n">
+        <v>-2.05</v>
+      </c>
+      <c r="I530" s="11" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average ($107.96) dropped below its 30-hour average ($108.85). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -20687,19 +20802,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>654.7</v>
+        <v>649.02</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>117.47</v>
+        <v>122.63</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>54.7</v>
+        <v>49.02</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>9.119999999999999</v>
+        <v>8.17</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -20709,19 +20824,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>574.4299999999999</v>
+        <v>572.38</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>376.62</v>
+        <v>484.44</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-25.57</v>
+        <v>-27.62</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.26</v>
+        <v>-4.6</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -20761,7 +20876,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-24 23:00 UTC</t>
+          <t>Generated: 2026-09-25 17:39 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-28 19:55 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I530"/>
+  <dimension ref="A1:I535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20715,6 +20715,197 @@
       <c r="I530" s="11" t="inlineStr">
         <is>
           <t>WMT's 10-hour average ($107.96) dropped below its 30-hour average ($108.85). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="531" ht="40" customHeight="1">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:55</t>
+        </is>
+      </c>
+      <c r="B531" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C531" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E531" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F531" s="2" t="n">
+        <v>108.81</v>
+      </c>
+      <c r="G531" s="2" t="n">
+        <v>108.81</v>
+      </c>
+      <c r="H531" s="2" t="inlineStr"/>
+      <c r="I531" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 0.95% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="532" ht="40" customHeight="1">
+      <c r="A532" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:55</t>
+        </is>
+      </c>
+      <c r="B532" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C532" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D532" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E532" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F532" s="8" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="G532" s="8" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="H532" s="10" t="n">
+        <v>-8.19</v>
+      </c>
+      <c r="I532" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: NFLX dropped 10.6% from the entry price (bought at $77.26, now $69.07). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="533" ht="40" customHeight="1">
+      <c r="A533" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:55</t>
+        </is>
+      </c>
+      <c r="B533" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C533" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D533" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E533" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F533" s="8" t="n">
+        <v>108.81</v>
+      </c>
+      <c r="G533" s="8" t="n">
+        <v>108.81</v>
+      </c>
+      <c r="H533" s="12" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I533" s="11" t="inlineStr">
+        <is>
+          <t>WMT's RSI climbed to 73.1, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="534" ht="40" customHeight="1">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:55</t>
+        </is>
+      </c>
+      <c r="B534" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C534" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E534" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F534" s="2" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="G534" s="2" t="n">
+        <v>69.06999999999999</v>
+      </c>
+      <c r="H534" s="2" t="inlineStr"/>
+      <c r="I534" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's RSI is 11.3, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="535" ht="40" customHeight="1">
+      <c r="A535" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-28 19:55</t>
+        </is>
+      </c>
+      <c r="B535" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C535" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D535" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E535" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F535" s="8" t="n">
+        <v>87.33</v>
+      </c>
+      <c r="G535" s="8" t="n">
+        <v>87.33</v>
+      </c>
+      <c r="H535" s="10" t="n">
+        <v>-0.6</v>
+      </c>
+      <c r="I535" s="11" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average ($87.43) dropped below its 30-hour average ($88.01). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -20783,7 +20974,7 @@
         <v>624.17</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>624.17</v>
+        <v>515.37</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -20802,19 +20993,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>649.02</v>
+        <v>641.8099999999999</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>122.63</v>
+        <v>231.44</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>49.02</v>
+        <v>41.81</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>8.17</v>
+        <v>6.97</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -20824,19 +21015,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>572.38</v>
+        <v>571.78</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>484.44</v>
+        <v>571.78</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-27.62</v>
+        <v>-28.22</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.6</v>
+        <v>-4.7</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -20876,7 +21067,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-25 23:05 UTC</t>
+          <t>Generated: 2026-09-28 19:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-29 18:23 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I535"/>
+  <dimension ref="A1:I540"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -20906,6 +20906,195 @@
       <c r="I535" s="11" t="inlineStr">
         <is>
           <t>KO's 10-hour average ($87.43) dropped below its 30-hour average ($88.01). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="536" ht="40" customHeight="1">
+      <c r="A536" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:23</t>
+        </is>
+      </c>
+      <c r="B536" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C536" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D536" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E536" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F536" s="8" t="n">
+        <v>106.53</v>
+      </c>
+      <c r="G536" s="8" t="n">
+        <v>106.53</v>
+      </c>
+      <c r="H536" s="10" t="n">
+        <v>-2.28</v>
+      </c>
+      <c r="I536" s="11" t="inlineStr">
+        <is>
+          <t>WMT lost momentum: down 2.31% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="537" ht="40" customHeight="1">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:23</t>
+        </is>
+      </c>
+      <c r="B537" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C537" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E537" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F537" s="2" t="n">
+        <v>70.20999999999999</v>
+      </c>
+      <c r="G537" s="2" t="n">
+        <v>70.20999999999999</v>
+      </c>
+      <c r="H537" s="2" t="inlineStr"/>
+      <c r="I537" s="4" t="inlineStr">
+        <is>
+          <t>NFLX is ranked #3 out of 25 stocks by momentum. It gained 1.09% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="538" ht="40" customHeight="1">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:23</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C538" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E538" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F538" s="2" t="n">
+        <v>128.56</v>
+      </c>
+      <c r="G538" s="2" t="n">
+        <v>128.56</v>
+      </c>
+      <c r="H538" s="2" t="inlineStr"/>
+      <c r="I538" s="4" t="inlineStr">
+        <is>
+          <t>PEP is ranked #4 out of 25 stocks by momentum. It gained 0.81% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="539" ht="40" customHeight="1">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:23</t>
+        </is>
+      </c>
+      <c r="B539" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C539" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E539" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F539" s="2" t="n">
+        <v>55.06</v>
+      </c>
+      <c r="G539" s="2" t="n">
+        <v>110.12</v>
+      </c>
+      <c r="H539" s="2" t="inlineStr"/>
+      <c r="I539" s="4" t="inlineStr">
+        <is>
+          <t>BAC's RSI is 21.2, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="540" ht="40" customHeight="1">
+      <c r="A540" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-29 18:23</t>
+        </is>
+      </c>
+      <c r="B540" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C540" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D540" s="8" t="inlineStr">
+        <is>
+          <t>T</t>
+        </is>
+      </c>
+      <c r="E540" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="F540" s="8" t="n">
+        <v>24.64</v>
+      </c>
+      <c r="G540" s="8" t="n">
+        <v>98.54000000000001</v>
+      </c>
+      <c r="H540" s="10" t="n">
+        <v>-8.880000000000001</v>
+      </c>
+      <c r="I540" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: T dropped 8.3% from the entry price (bought at $26.85, now $24.64). Selling automatically to protect capital before losses grow further.</t>
         </is>
       </c>
     </row>
@@ -20971,19 +21160,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>624.17</v>
+        <v>621.9</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>515.37</v>
+        <v>423.12</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>24.17</v>
+        <v>21.9</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.03</v>
+        <v>3.65</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -20996,7 +21185,7 @@
         <v>641.8099999999999</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>231.44</v>
+        <v>121.32</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
@@ -21037,19 +21226,19 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>556.84</v>
+        <v>547.96</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>59.23</v>
+        <v>157.77</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-43.16</v>
+        <v>-52.04</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-7.19</v>
+        <v>-8.67</v>
       </c>
     </row>
     <row r="6">
@@ -21067,7 +21256,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-29 00:12 UTC</t>
+          <t>Generated: 2026-09-29 18:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-09-30 18:13 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I540"/>
+  <dimension ref="A1:I544"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21095,6 +21095,158 @@
       <c r="I540" s="11" t="inlineStr">
         <is>
           <t>STOP-LOSS: T dropped 8.3% from the entry price (bought at $26.85, now $24.64). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="541" ht="40" customHeight="1">
+      <c r="A541" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:13</t>
+        </is>
+      </c>
+      <c r="B541" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C541" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D541" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E541" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F541" s="8" t="n">
+        <v>69.79000000000001</v>
+      </c>
+      <c r="G541" s="8" t="n">
+        <v>69.79000000000001</v>
+      </c>
+      <c r="H541" s="10" t="n">
+        <v>-0.43</v>
+      </c>
+      <c r="I541" s="11" t="inlineStr">
+        <is>
+          <t>NFLX lost momentum: down 0.94% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="542" ht="40" customHeight="1">
+      <c r="A542" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:13</t>
+        </is>
+      </c>
+      <c r="B542" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C542" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D542" s="8" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E542" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F542" s="8" t="n">
+        <v>127.43</v>
+      </c>
+      <c r="G542" s="8" t="n">
+        <v>127.43</v>
+      </c>
+      <c r="H542" s="10" t="n">
+        <v>-1.12</v>
+      </c>
+      <c r="I542" s="11" t="inlineStr">
+        <is>
+          <t>PEP lost momentum: down 0.31% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="543" ht="40" customHeight="1">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:13</t>
+        </is>
+      </c>
+      <c r="B543" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C543" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E543" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F543" s="2" t="n">
+        <v>105.18</v>
+      </c>
+      <c r="G543" s="2" t="n">
+        <v>105.18</v>
+      </c>
+      <c r="H543" s="2" t="inlineStr"/>
+      <c r="I543" s="4" t="inlineStr">
+        <is>
+          <t>WMT's RSI is 22.6, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="544" ht="40" customHeight="1">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-30 18:13</t>
+        </is>
+      </c>
+      <c r="B544" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C544" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>NEE</t>
+        </is>
+      </c>
+      <c r="E544" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F544" s="2" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="G544" s="2" t="n">
+        <v>76.15000000000001</v>
+      </c>
+      <c r="H544" s="2" t="inlineStr"/>
+      <c r="I544" s="4" t="inlineStr">
+        <is>
+          <t>NEE pays a 3.28% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($76.15) is above its 30-hour average ($75.82), confirming a healthy trend. Buying to collect steady income while holding.</t>
         </is>
       </c>
     </row>
@@ -21160,19 +21312,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>621.9</v>
+        <v>620.34</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>423.12</v>
+        <v>620.34</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>21.9</v>
+        <v>20.34</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>3.65</v>
+        <v>3.39</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -21185,7 +21337,7 @@
         <v>641.8099999999999</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>121.32</v>
+        <v>16.14</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
@@ -21229,7 +21381,7 @@
         <v>547.96</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>157.77</v>
+        <v>81.62</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
@@ -21256,7 +21408,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-09-29 23:27 UTC</t>
+          <t>Generated: 2026-09-30 18:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-06 18:42 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I544"/>
+  <dimension ref="A1:I552"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21247,6 +21247,306 @@
       <c r="I544" s="4" t="inlineStr">
         <is>
           <t>NEE pays a 3.28% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($76.15) is above its 30-hour average ($75.82), confirming a healthy trend. Buying to collect steady income while holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="545" ht="40" customHeight="1">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C545" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E545" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F545" s="2" t="n">
+        <v>68.23999999999999</v>
+      </c>
+      <c r="G545" s="2" t="n">
+        <v>68.23999999999999</v>
+      </c>
+      <c r="H545" s="2" t="inlineStr"/>
+      <c r="I545" s="4" t="inlineStr">
+        <is>
+          <t>NFLX is ranked #2 out of 25 stocks by momentum. It gained 2.28% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="546" ht="40" customHeight="1">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B546" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C546" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E546" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F546" s="2" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="G546" s="2" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="H546" s="2" t="inlineStr"/>
+      <c r="I546" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #3 out of 25 stocks by momentum. It gained 2.18% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="547" ht="40" customHeight="1">
+      <c r="A547" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B547" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C547" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D547" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E547" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F547" s="8" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="G547" s="8" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="H547" s="12" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="I547" s="11" t="inlineStr">
+        <is>
+          <t>WMT's RSI climbed to 90.2, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="548" ht="40" customHeight="1">
+      <c r="A548" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B548" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C548" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D548" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E548" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F548" s="8" t="n">
+        <v>68.23999999999999</v>
+      </c>
+      <c r="G548" s="8" t="n">
+        <v>68.23999999999999</v>
+      </c>
+      <c r="H548" s="10" t="n">
+        <v>-0.83</v>
+      </c>
+      <c r="I548" s="11" t="inlineStr">
+        <is>
+          <t>NFLX's RSI climbed to 67.8, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="549" ht="40" customHeight="1">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B549" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C549" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E549" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F549" s="2" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="G549" s="2" t="n">
+        <v>106.96</v>
+      </c>
+      <c r="H549" s="2" t="inlineStr"/>
+      <c r="I549" s="4" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average price ($105.93) is above its 30-hour average ($104.93). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="550" ht="40" customHeight="1">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B550" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C550" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E550" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F550" s="2" t="n">
+        <v>54.1</v>
+      </c>
+      <c r="G550" s="2" t="n">
+        <v>108.19</v>
+      </c>
+      <c r="H550" s="2" t="inlineStr"/>
+      <c r="I550" s="4" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average price ($54.15) is above its 30-hour average ($53.91). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="551" ht="40" customHeight="1">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B551" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C551" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E551" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F551" s="2" t="n">
+        <v>86.79000000000001</v>
+      </c>
+      <c r="G551" s="2" t="n">
+        <v>86.79000000000001</v>
+      </c>
+      <c r="H551" s="2" t="inlineStr"/>
+      <c r="I551" s="4" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average price ($86.72) is above its 30-hour average ($86.22). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="552" ht="40" customHeight="1">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-06 18:42</t>
+        </is>
+      </c>
+      <c r="B552" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C552" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="E552" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F552" s="2" t="n">
+        <v>54.01</v>
+      </c>
+      <c r="G552" s="2" t="n">
+        <v>54.01</v>
+      </c>
+      <c r="H552" s="2" t="inlineStr"/>
+      <c r="I552" s="4" t="inlineStr">
+        <is>
+          <t>O pays a 6.06% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($54.01) is above its 30-hour average ($53.97), confirming a healthy trend. Buying to collect steady income while holding.</t>
         </is>
       </c>
     </row>
@@ -21315,7 +21615,7 @@
         <v>620.34</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>620.34</v>
+        <v>445.15</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -21334,19 +21634,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>641.8099999999999</v>
+        <v>642.75</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>16.14</v>
+        <v>191.33</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>41.81</v>
+        <v>42.75</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>6.97</v>
+        <v>7.13</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -21359,7 +21659,7 @@
         <v>571.78</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>571.78</v>
+        <v>269.85</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -21381,7 +21681,7 @@
         <v>547.96</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>81.62</v>
+        <v>27.61</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
@@ -21408,7 +21708,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-06 01:07 UTC</t>
+          <t>Generated: 2026-10-06 18:42 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-07 19:08 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I552"/>
+  <dimension ref="A1:I555"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21547,6 +21547,121 @@
       <c r="I552" s="4" t="inlineStr">
         <is>
           <t>O pays a 6.06% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($54.01) is above its 30-hour average ($53.97), confirming a healthy trend. Buying to collect steady income while holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="553" ht="40" customHeight="1">
+      <c r="A553" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:08</t>
+        </is>
+      </c>
+      <c r="B553" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C553" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D553" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E553" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F553" s="8" t="n">
+        <v>108.28</v>
+      </c>
+      <c r="G553" s="8" t="n">
+        <v>108.28</v>
+      </c>
+      <c r="H553" s="12" t="n">
+        <v>1.32</v>
+      </c>
+      <c r="I553" s="11" t="inlineStr">
+        <is>
+          <t>WMT dropped out of the top 5 momentum stocks (current momentum: 1.37%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="554" ht="40" customHeight="1">
+      <c r="A554" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:08</t>
+        </is>
+      </c>
+      <c r="B554" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C554" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D554" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E554" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F554" s="8" t="n">
+        <v>53.37</v>
+      </c>
+      <c r="G554" s="8" t="n">
+        <v>106.73</v>
+      </c>
+      <c r="H554" s="10" t="n">
+        <v>-1.46</v>
+      </c>
+      <c r="I554" s="11" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average ($53.67) dropped below its 30-hour average ($53.84). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="555" ht="40" customHeight="1">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-07 19:08</t>
+        </is>
+      </c>
+      <c r="B555" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C555" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E555" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F555" s="2" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="G555" s="2" t="n">
+        <v>69.59999999999999</v>
+      </c>
+      <c r="H555" s="2" t="inlineStr"/>
+      <c r="I555" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average price ($68.82) is above its 30-hour average ($67.85). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -21612,19 +21727,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>620.34</v>
+        <v>621.67</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>445.15</v>
+        <v>553.4299999999999</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>20.34</v>
+        <v>21.67</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>3.39</v>
+        <v>3.61</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -21656,19 +21771,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>571.78</v>
+        <v>570.3200000000001</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>269.85</v>
+        <v>306.98</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-28.22</v>
+        <v>-29.68</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.7</v>
+        <v>-4.95</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -21708,7 +21823,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-06 23:34 UTC</t>
+          <t>Generated: 2026-10-07 19:08 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-08 19:04 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I555"/>
+  <dimension ref="A1:I558"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21662,6 +21662,119 @@
       <c r="I555" s="4" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average price ($68.82) is above its 30-hour average ($67.85). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="556" ht="40" customHeight="1">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 19:04</t>
+        </is>
+      </c>
+      <c r="B556" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C556" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E556" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F556" s="2" t="n">
+        <v>110.96</v>
+      </c>
+      <c r="G556" s="2" t="n">
+        <v>110.96</v>
+      </c>
+      <c r="H556" s="2" t="inlineStr"/>
+      <c r="I556" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 2.20% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="557" ht="40" customHeight="1">
+      <c r="A557" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-08 19:04</t>
+        </is>
+      </c>
+      <c r="B557" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C557" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D557" s="8" t="inlineStr">
+        <is>
+          <t>CVX</t>
+        </is>
+      </c>
+      <c r="E557" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F557" s="8" t="n">
+        <v>211.94</v>
+      </c>
+      <c r="G557" s="8" t="n">
+        <v>211.94</v>
+      </c>
+      <c r="H557" s="12" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I557" s="11" t="inlineStr">
+        <is>
+          <t>CVX's RSI climbed to 65.8, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="558" ht="40" customHeight="1">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-08 19:04</t>
+        </is>
+      </c>
+      <c r="B558" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C558" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="E558" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F558" s="2" t="n">
+        <v>150.38</v>
+      </c>
+      <c r="G558" s="2" t="n">
+        <v>150.38</v>
+      </c>
+      <c r="H558" s="2" t="inlineStr"/>
+      <c r="I558" s="4" t="inlineStr">
+        <is>
+          <t>PG's 10-hour average price ($148.98) is above its 30-hour average ($147.69). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -21730,7 +21843,7 @@
         <v>621.67</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>553.4299999999999</v>
+        <v>442.48</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -21749,19 +21862,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>642.75</v>
+        <v>643.65</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>191.33</v>
+        <v>403.27</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>42.75</v>
+        <v>43.65</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>7.13</v>
+        <v>7.28</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -21774,7 +21887,7 @@
         <v>570.3200000000001</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>306.98</v>
+        <v>156.6</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -21823,7 +21936,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-08 00:00 UTC</t>
+          <t>Generated: 2026-10-08 19:04 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-09 18:35 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I558"/>
+  <dimension ref="A1:I564"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -21775,6 +21775,234 @@
       <c r="I558" s="4" t="inlineStr">
         <is>
           <t>PG's 10-hour average price ($148.98) is above its 30-hour average ($147.69). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="559" ht="40" customHeight="1">
+      <c r="A559" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B559" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C559" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D559" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E559" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F559" s="8" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="G559" s="8" t="n">
+        <v>70.5</v>
+      </c>
+      <c r="H559" s="12" t="n">
+        <v>2.27</v>
+      </c>
+      <c r="I559" s="11" t="inlineStr">
+        <is>
+          <t>NFLX lost momentum: down 0.82% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="560" ht="40" customHeight="1">
+      <c r="A560" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B560" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C560" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D560" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E560" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F560" s="8" t="n">
+        <v>111.34</v>
+      </c>
+      <c r="G560" s="8" t="n">
+        <v>111.34</v>
+      </c>
+      <c r="H560" s="12" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I560" s="11" t="inlineStr">
+        <is>
+          <t>WMT dropped out of the top 5 momentum stocks (current momentum: 0.96%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="561" ht="40" customHeight="1">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C561" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E561" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F561" s="2" t="n">
+        <v>54.26</v>
+      </c>
+      <c r="G561" s="2" t="n">
+        <v>108.51</v>
+      </c>
+      <c r="H561" s="2" t="inlineStr"/>
+      <c r="I561" s="4" t="inlineStr">
+        <is>
+          <t>BAC is ranked #3 out of 25 stocks by momentum. It gained 3.35% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="562" ht="40" customHeight="1">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B562" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C562" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E562" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F562" s="2" t="n">
+        <v>54.26</v>
+      </c>
+      <c r="G562" s="2" t="n">
+        <v>108.51</v>
+      </c>
+      <c r="H562" s="2" t="inlineStr"/>
+      <c r="I562" s="4" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average price ($53.72) is above its 30-hour average ($53.68). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="563" ht="40" customHeight="1">
+      <c r="A563" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B563" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C563" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D563" s="8" t="inlineStr">
+        <is>
+          <t>VZ</t>
+        </is>
+      </c>
+      <c r="E563" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="F563" s="8" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="G563" s="8" t="n">
+        <v>123.9</v>
+      </c>
+      <c r="H563" s="10" t="n">
+        <v>-21.36</v>
+      </c>
+      <c r="I563" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: VZ dropped 14.7% from the entry price (bought at $48.42, now $41.30). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="564" ht="40" customHeight="1">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-09 18:35</t>
+        </is>
+      </c>
+      <c r="B564" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C564" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E564" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F564" s="2" t="n">
+        <v>126.07</v>
+      </c>
+      <c r="G564" s="2" t="n">
+        <v>126.07</v>
+      </c>
+      <c r="H564" s="2" t="inlineStr"/>
+      <c r="I564" s="4" t="inlineStr">
+        <is>
+          <t>PEP pays a 4.61% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($126.07) is above its 30-hour average ($125.65), confirming a healthy trend. Buying to collect steady income while holding.</t>
         </is>
       </c>
     </row>
@@ -21840,19 +22068,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>621.67</v>
+        <v>624.3200000000001</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>442.48</v>
+        <v>515.8099999999999</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>21.67</v>
+        <v>24.32</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>3.61</v>
+        <v>4.05</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -21887,7 +22115,7 @@
         <v>570.3200000000001</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>156.6</v>
+        <v>48.09</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -21906,19 +22134,19 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>547.96</v>
+        <v>526.6</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>27.61</v>
+        <v>25.43</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-52.04</v>
+        <v>-73.40000000000001</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-8.67</v>
+        <v>-12.23</v>
       </c>
     </row>
     <row r="6">
@@ -21936,7 +22164,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-09 00:08 UTC</t>
+          <t>Generated: 2026-10-09 18:35 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-13 19:40 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I564"/>
+  <dimension ref="A1:I567"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22003,6 +22003,121 @@
       <c r="I564" s="4" t="inlineStr">
         <is>
           <t>PEP pays a 4.61% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($126.07) is above its 30-hour average ($125.65), confirming a healthy trend. Buying to collect steady income while holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="565" ht="40" customHeight="1">
+      <c r="A565" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:40</t>
+        </is>
+      </c>
+      <c r="B565" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C565" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D565" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E565" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F565" s="8" t="n">
+        <v>54.18</v>
+      </c>
+      <c r="G565" s="8" t="n">
+        <v>108.36</v>
+      </c>
+      <c r="H565" s="10" t="n">
+        <v>-0.15</v>
+      </c>
+      <c r="I565" s="11" t="inlineStr">
+        <is>
+          <t>BAC lost momentum: down 0.43% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="566" ht="40" customHeight="1">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:40</t>
+        </is>
+      </c>
+      <c r="B566" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C566" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E566" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F566" s="2" t="n">
+        <v>90.31999999999999</v>
+      </c>
+      <c r="G566" s="2" t="n">
+        <v>90.31999999999999</v>
+      </c>
+      <c r="H566" s="2" t="inlineStr"/>
+      <c r="I566" s="4" t="inlineStr">
+        <is>
+          <t>KO is ranked #5 out of 25 stocks by momentum. It gained 1.16% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="567" ht="40" customHeight="1">
+      <c r="A567" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-13 19:40</t>
+        </is>
+      </c>
+      <c r="B567" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C567" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D567" s="8" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E567" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F567" s="8" t="n">
+        <v>127.42</v>
+      </c>
+      <c r="G567" s="8" t="n">
+        <v>127.42</v>
+      </c>
+      <c r="H567" s="10" t="n">
+        <v>-2.84</v>
+      </c>
+      <c r="I567" s="11" t="inlineStr">
+        <is>
+          <t>PEP's RSI climbed to 67.6, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
         </is>
       </c>
     </row>
@@ -22068,19 +22183,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>624.3200000000001</v>
+        <v>624.17</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>515.8099999999999</v>
+        <v>533.85</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>24.32</v>
+        <v>24.17</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.05</v>
+        <v>4.03</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -22090,19 +22205,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>643.65</v>
+        <v>640.8099999999999</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>403.27</v>
+        <v>530.6900000000001</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>43.65</v>
+        <v>40.81</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>7.28</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -22164,7 +22279,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-13 01:49 UTC</t>
+          <t>Generated: 2026-10-13 19:40 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-14 17:41 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I567"/>
+  <dimension ref="A1:I570"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22118,6 +22118,121 @@
       <c r="I567" s="11" t="inlineStr">
         <is>
           <t>PEP's RSI climbed to 67.6, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="568" ht="40" customHeight="1">
+      <c r="A568" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:41</t>
+        </is>
+      </c>
+      <c r="B568" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C568" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D568" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E568" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F568" s="8" t="n">
+        <v>50.67</v>
+      </c>
+      <c r="G568" s="8" t="n">
+        <v>101.34</v>
+      </c>
+      <c r="H568" s="10" t="n">
+        <v>-7.17</v>
+      </c>
+      <c r="I568" s="11" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average ($52.25) dropped below its 30-hour average ($53.46). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="569" ht="40" customHeight="1">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:41</t>
+        </is>
+      </c>
+      <c r="B569" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C569" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="E569" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F569" s="2" t="n">
+        <v>147.91</v>
+      </c>
+      <c r="G569" s="2" t="n">
+        <v>147.91</v>
+      </c>
+      <c r="H569" s="2" t="inlineStr"/>
+      <c r="I569" s="4" t="inlineStr">
+        <is>
+          <t>MRK's 10-hour average price ($144.59) is above its 30-hour average ($144.57). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="570" ht="40" customHeight="1">
+      <c r="A570" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-14 17:41</t>
+        </is>
+      </c>
+      <c r="B570" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C570" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D570" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E570" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F570" s="8" t="n">
+        <v>70.11</v>
+      </c>
+      <c r="G570" s="8" t="n">
+        <v>70.11</v>
+      </c>
+      <c r="H570" s="12" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="I570" s="11" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average ($70.32) dropped below its 30-hour average ($70.71). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -22227,19 +22342,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>570.3200000000001</v>
+        <v>563.67</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>48.09</v>
+        <v>71.64</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-29.68</v>
+        <v>-36.33</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.95</v>
+        <v>-6.06</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -22279,7 +22394,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-13 23:36 UTC</t>
+          <t>Generated: 2026-10-14 17:41 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-15 17:31 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I570"/>
+  <dimension ref="A1:I574"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22233,6 +22233,156 @@
       <c r="I570" s="11" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average ($70.32) dropped below its 30-hour average ($70.71). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="571" ht="40" customHeight="1">
+      <c r="A571" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-15 17:31</t>
+        </is>
+      </c>
+      <c r="B571" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C571" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D571" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E571" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F571" s="8" t="n">
+        <v>92.36</v>
+      </c>
+      <c r="G571" s="8" t="n">
+        <v>92.36</v>
+      </c>
+      <c r="H571" s="12" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="I571" s="11" t="inlineStr">
+        <is>
+          <t>KO dropped out of the top 5 momentum stocks (current momentum: 1.08%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="572" ht="40" customHeight="1">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 17:31</t>
+        </is>
+      </c>
+      <c r="B572" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C572" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E572" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F572" s="2" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="G572" s="2" t="n">
+        <v>72.67</v>
+      </c>
+      <c r="H572" s="2" t="inlineStr"/>
+      <c r="I572" s="4" t="inlineStr">
+        <is>
+          <t>NFLX is ranked #2 out of 25 stocks by momentum. It gained 4.62% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="573" ht="40" customHeight="1">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 17:31</t>
+        </is>
+      </c>
+      <c r="B573" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C573" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E573" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F573" s="2" t="n">
+        <v>51.97</v>
+      </c>
+      <c r="G573" s="2" t="n">
+        <v>103.93</v>
+      </c>
+      <c r="H573" s="2" t="inlineStr"/>
+      <c r="I573" s="4" t="inlineStr">
+        <is>
+          <t>BAC is ranked #4 out of 25 stocks by momentum. It gained 3.44% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="574" ht="40" customHeight="1">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-15 17:31</t>
+        </is>
+      </c>
+      <c r="B574" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C574" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E574" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F574" s="2" t="n">
+        <v>118.53</v>
+      </c>
+      <c r="G574" s="2" t="n">
+        <v>118.53</v>
+      </c>
+      <c r="H574" s="2" t="inlineStr"/>
+      <c r="I574" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 3.29% over the last 10 hours, showing strong upward price pressure.</t>
         </is>
       </c>
     </row>
@@ -22298,19 +22448,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>624.17</v>
+        <v>626.21</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>533.85</v>
+        <v>331.08</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>24.17</v>
+        <v>26.21</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.03</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -22394,7 +22544,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-14 22:59 UTC</t>
+          <t>Generated: 2026-10-15 17:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-16 17:06 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I574"/>
+  <dimension ref="A1:I578"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22383,6 +22383,160 @@
       <c r="I574" s="4" t="inlineStr">
         <is>
           <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 3.29% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="575" ht="40" customHeight="1">
+      <c r="A575" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:06</t>
+        </is>
+      </c>
+      <c r="B575" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C575" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D575" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E575" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F575" s="8" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="G575" s="8" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="H575" s="10" t="n">
+        <v>-2.07</v>
+      </c>
+      <c r="I575" s="11" t="inlineStr">
+        <is>
+          <t>NFLX lost momentum: down 2.44% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="576" ht="40" customHeight="1">
+      <c r="A576" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:06</t>
+        </is>
+      </c>
+      <c r="B576" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C576" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D576" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E576" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F576" s="8" t="n">
+        <v>51.62</v>
+      </c>
+      <c r="G576" s="8" t="n">
+        <v>103.24</v>
+      </c>
+      <c r="H576" s="10" t="n">
+        <v>-0.6899999999999999</v>
+      </c>
+      <c r="I576" s="11" t="inlineStr">
+        <is>
+          <t>BAC dropped out of the top 5 momentum stocks (current momentum: 0.61%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="577" ht="40" customHeight="1">
+      <c r="A577" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:06</t>
+        </is>
+      </c>
+      <c r="B577" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C577" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D577" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E577" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F577" s="8" t="n">
+        <v>118.71</v>
+      </c>
+      <c r="G577" s="8" t="n">
+        <v>118.71</v>
+      </c>
+      <c r="H577" s="12" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I577" s="11" t="inlineStr">
+        <is>
+          <t>WMT lost momentum: down 1.51% over the last 10 hours. Selling to avoid further losses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="578" ht="40" customHeight="1">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 17:06</t>
+        </is>
+      </c>
+      <c r="B578" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C578" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E578" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F578" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="G578" s="2" t="n">
+        <v>70.61</v>
+      </c>
+      <c r="H578" s="2" t="inlineStr"/>
+      <c r="I578" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average price ($71.91) is above its 30-hour average ($71.07). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -22448,19 +22602,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>626.21</v>
+        <v>623.63</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>331.08</v>
+        <v>623.63</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>26.21</v>
+        <v>23.63</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>4.37</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -22495,7 +22649,7 @@
         <v>563.67</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>71.64</v>
+        <v>1.03</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -22544,7 +22698,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-15 22:54 UTC</t>
+          <t>Generated: 2026-10-16 17:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-16 19:55 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I578"/>
+  <dimension ref="A1:I579"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22537,6 +22537,43 @@
       <c r="I578" s="4" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average price ($71.91) is above its 30-hour average ($71.07). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="579" ht="40" customHeight="1">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16 19:54</t>
+        </is>
+      </c>
+      <c r="B579" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C579" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E579" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F579" s="2" t="n">
+        <v>93.45999999999999</v>
+      </c>
+      <c r="G579" s="2" t="n">
+        <v>93.45999999999999</v>
+      </c>
+      <c r="H579" s="2" t="inlineStr"/>
+      <c r="I579" s="4" t="inlineStr">
+        <is>
+          <t>KO is ranked #5 out of 25 stocks by momentum. It gained 1.14% over the last 10 hours, showing strong upward price pressure.</t>
         </is>
       </c>
     </row>
@@ -22605,7 +22642,7 @@
         <v>623.63</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>623.63</v>
+        <v>530.17</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -22698,7 +22735,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-16 17:06 UTC</t>
+          <t>Generated: 2026-10-16 19:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-19 18:55 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I579"/>
+  <dimension ref="A1:I586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22574,6 +22574,273 @@
       <c r="I579" s="4" t="inlineStr">
         <is>
           <t>KO is ranked #5 out of 25 stocks by momentum. It gained 1.14% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="580" ht="40" customHeight="1">
+      <c r="A580" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B580" s="9" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C580" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D580" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E580" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F580" s="8" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="G580" s="8" t="n">
+        <v>93.75</v>
+      </c>
+      <c r="H580" s="12" t="n">
+        <v>0.29</v>
+      </c>
+      <c r="I580" s="11" t="inlineStr">
+        <is>
+          <t>KO dropped out of the top 5 momentum stocks (current momentum: 0.51%). Rotating into stronger performers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="581" ht="40" customHeight="1">
+      <c r="A581" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B581" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C581" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D581" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E581" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F581" s="8" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G581" s="8" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="H581" s="10" t="n">
+        <v>-9.32</v>
+      </c>
+      <c r="I581" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: BAC dropped 8.5% from the entry price (bought at $55.06, now $50.40). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="582" ht="40" customHeight="1">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B582" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C582" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E582" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F582" s="2" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G582" s="2" t="n">
+        <v>100.8</v>
+      </c>
+      <c r="H582" s="2" t="inlineStr"/>
+      <c r="I582" s="4" t="inlineStr">
+        <is>
+          <t>BAC's RSI is 28.7, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="583" ht="40" customHeight="1">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B583" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C583" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E583" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F583" s="2" t="n">
+        <v>69.70999999999999</v>
+      </c>
+      <c r="G583" s="2" t="n">
+        <v>69.70999999999999</v>
+      </c>
+      <c r="H583" s="2" t="inlineStr"/>
+      <c r="I583" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's RSI is 15.2, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="584" ht="40" customHeight="1">
+      <c r="A584" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B584" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C584" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D584" s="8" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="E584" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F584" s="8" t="n">
+        <v>144.02</v>
+      </c>
+      <c r="G584" s="8" t="n">
+        <v>144.02</v>
+      </c>
+      <c r="H584" s="10" t="n">
+        <v>-3.89</v>
+      </c>
+      <c r="I584" s="11" t="inlineStr">
+        <is>
+          <t>MRK's 10-hour average ($145.45) dropped below its 30-hour average ($146.25). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="585" ht="40" customHeight="1">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B585" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C585" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E585" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F585" s="2" t="n">
+        <v>133.45</v>
+      </c>
+      <c r="G585" s="2" t="n">
+        <v>133.45</v>
+      </c>
+      <c r="H585" s="2" t="inlineStr"/>
+      <c r="I585" s="4" t="inlineStr">
+        <is>
+          <t>PEP's 10-hour average price ($132.07) is above its 30-hour average ($130.20). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="586" ht="40" customHeight="1">
+      <c r="A586" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-19 18:55</t>
+        </is>
+      </c>
+      <c r="B586" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C586" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D586" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E586" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F586" s="8" t="n">
+        <v>69.70999999999999</v>
+      </c>
+      <c r="G586" s="8" t="n">
+        <v>69.70999999999999</v>
+      </c>
+      <c r="H586" s="10" t="n">
+        <v>-0.89</v>
+      </c>
+      <c r="I586" s="11" t="inlineStr">
+        <is>
+          <t>NFLX's 10-hour average ($69.91) dropped below its 30-hour average ($70.76). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -22639,19 +22906,19 @@
         </is>
       </c>
       <c r="B2" s="16" t="n">
-        <v>623.63</v>
+        <v>623.92</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>530.17</v>
+        <v>623.92</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E2" s="17" t="n">
-        <v>23.63</v>
+        <v>23.92</v>
       </c>
       <c r="F2" s="17" t="n">
-        <v>3.94</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
@@ -22661,19 +22928,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>640.8099999999999</v>
+        <v>631.49</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>530.6900000000001</v>
+        <v>460.98</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>40.81</v>
+        <v>31.49</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>6.8</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -22683,19 +22950,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>563.67</v>
+        <v>558.89</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>1.03</v>
+        <v>81.31999999999999</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-36.33</v>
+        <v>-41.11</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-6.06</v>
+        <v>-6.85</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -22735,7 +23002,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-16 22:32 UTC</t>
+          <t>Generated: 2026-10-19 18:55 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-21 17:47 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I586"/>
+  <dimension ref="A1:I590"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22841,6 +22841,158 @@
       <c r="I586" s="11" t="inlineStr">
         <is>
           <t>NFLX's 10-hour average ($69.91) dropped below its 30-hour average ($70.76). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="587" ht="40" customHeight="1">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47</t>
+        </is>
+      </c>
+      <c r="B587" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C587" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E587" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F587" s="2" t="n">
+        <v>117.91</v>
+      </c>
+      <c r="G587" s="2" t="n">
+        <v>117.91</v>
+      </c>
+      <c r="H587" s="2" t="inlineStr"/>
+      <c r="I587" s="4" t="inlineStr">
+        <is>
+          <t>WMT's RSI is 34.1, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="588" ht="40" customHeight="1">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47</t>
+        </is>
+      </c>
+      <c r="B588" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C588" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E588" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F588" s="2" t="n">
+        <v>92.68000000000001</v>
+      </c>
+      <c r="G588" s="2" t="n">
+        <v>92.68000000000001</v>
+      </c>
+      <c r="H588" s="2" t="inlineStr"/>
+      <c r="I588" s="4" t="inlineStr">
+        <is>
+          <t>KO's RSI is 32.4, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="589" ht="40" customHeight="1">
+      <c r="A589" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47</t>
+        </is>
+      </c>
+      <c r="B589" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C589" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D589" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E589" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F589" s="8" t="n">
+        <v>117.91</v>
+      </c>
+      <c r="G589" s="8" t="n">
+        <v>117.91</v>
+      </c>
+      <c r="H589" s="12" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="I589" s="11" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average ($117.97) dropped below its 30-hour average ($118.43). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="590" ht="40" customHeight="1">
+      <c r="A590" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-21 17:47</t>
+        </is>
+      </c>
+      <c r="B590" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C590" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D590" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E590" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F590" s="8" t="n">
+        <v>92.68000000000001</v>
+      </c>
+      <c r="G590" s="8" t="n">
+        <v>92.68000000000001</v>
+      </c>
+      <c r="H590" s="12" t="n">
+        <v>5.89</v>
+      </c>
+      <c r="I590" s="11" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average ($92.95) dropped below its 30-hour average ($93.06). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -22931,7 +23083,7 @@
         <v>631.49</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>460.98</v>
+        <v>250.39</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
@@ -22950,19 +23102,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>558.89</v>
+        <v>575.73</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>81.31999999999999</v>
+        <v>291.91</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-41.11</v>
+        <v>-24.27</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-6.85</v>
+        <v>-4.04</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -23002,7 +23154,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-20 22:56 UTC</t>
+          <t>Generated: 2026-10-21 17:47 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-22 17:45 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I590"/>
+  <dimension ref="A1:I594"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -22993,6 +22993,158 @@
       <c r="I590" s="11" t="inlineStr">
         <is>
           <t>KO's 10-hour average ($92.95) dropped below its 30-hour average ($93.06). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="591" ht="40" customHeight="1">
+      <c r="A591" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:45</t>
+        </is>
+      </c>
+      <c r="B591" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C591" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D591" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E591" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F591" s="8" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="G591" s="8" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="H591" s="12" t="n">
+        <v>2.29</v>
+      </c>
+      <c r="I591" s="11" t="inlineStr">
+        <is>
+          <t>WMT's RSI climbed to 65.8, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="592" ht="40" customHeight="1">
+      <c r="A592" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:45</t>
+        </is>
+      </c>
+      <c r="B592" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C592" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D592" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E592" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F592" s="8" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="G592" s="8" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="H592" s="12" t="n">
+        <v>2.15</v>
+      </c>
+      <c r="I592" s="11" t="inlineStr">
+        <is>
+          <t>KO's RSI climbed to 74.6, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="593" ht="40" customHeight="1">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:45</t>
+        </is>
+      </c>
+      <c r="B593" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C593" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E593" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F593" s="2" t="n">
+        <v>50.94</v>
+      </c>
+      <c r="G593" s="2" t="n">
+        <v>50.94</v>
+      </c>
+      <c r="H593" s="2" t="inlineStr"/>
+      <c r="I593" s="4" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average price ($50.92) is above its 30-hour average ($50.89). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="594" ht="40" customHeight="1">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-22 17:45</t>
+        </is>
+      </c>
+      <c r="B594" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C594" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E594" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F594" s="2" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="G594" s="2" t="n">
+        <v>94.83</v>
+      </c>
+      <c r="H594" s="2" t="inlineStr"/>
+      <c r="I594" s="4" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average price ($93.72) is above its 30-hour average ($93.41). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -23080,19 +23232,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>631.49</v>
+        <v>635.9400000000001</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>250.39</v>
+        <v>465.42</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>31.49</v>
+        <v>35.94</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>5.25</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -23105,7 +23257,7 @@
         <v>575.73</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>291.91</v>
+        <v>146.14</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -23154,7 +23306,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-21 23:01 UTC</t>
+          <t>Generated: 2026-10-22 17:45 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-23 17:37 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I594"/>
+  <dimension ref="A1:I595"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23145,6 +23145,43 @@
       <c r="I594" s="4" t="inlineStr">
         <is>
           <t>KO's 10-hour average price ($93.72) is above its 30-hour average ($93.41). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="595" ht="40" customHeight="1">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-23 17:37</t>
+        </is>
+      </c>
+      <c r="B595" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C595" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E595" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F595" s="2" t="n">
+        <v>119.21</v>
+      </c>
+      <c r="G595" s="2" t="n">
+        <v>119.21</v>
+      </c>
+      <c r="H595" s="2" t="inlineStr"/>
+      <c r="I595" s="4" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average price ($120.15) is above its 30-hour average ($118.94). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -23257,7 +23294,7 @@
         <v>575.73</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>146.14</v>
+        <v>26.93</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -23306,7 +23343,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-22 22:58 UTC</t>
+          <t>Generated: 2026-10-23 17:37 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-26 18:57 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I595"/>
+  <dimension ref="A1:I602"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23182,6 +23182,275 @@
       <c r="I595" s="4" t="inlineStr">
         <is>
           <t>WMT's 10-hour average price ($120.15) is above its 30-hour average ($118.94). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="596" ht="40" customHeight="1">
+      <c r="A596" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B596" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C596" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D596" s="8" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E596" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F596" s="8" t="n">
+        <v>63.15</v>
+      </c>
+      <c r="G596" s="8" t="n">
+        <v>63.15</v>
+      </c>
+      <c r="H596" s="10" t="n">
+        <v>-6.56</v>
+      </c>
+      <c r="I596" s="11" t="inlineStr">
+        <is>
+          <t>STOP-LOSS: NFLX dropped 9.4% from the entry price (bought at $69.71, now $63.15). Selling automatically to protect capital before losses grow further.</t>
+        </is>
+      </c>
+    </row>
+    <row r="597" ht="40" customHeight="1">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B597" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C597" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E597" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F597" s="2" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="G597" s="2" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="H597" s="2" t="inlineStr"/>
+      <c r="I597" s="4" t="inlineStr">
+        <is>
+          <t>KO's RSI is 19.9, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="598" ht="40" customHeight="1">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B598" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C598" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>NFLX</t>
+        </is>
+      </c>
+      <c r="E598" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F598" s="2" t="n">
+        <v>63.15</v>
+      </c>
+      <c r="G598" s="2" t="n">
+        <v>126.31</v>
+      </c>
+      <c r="H598" s="2" t="inlineStr"/>
+      <c r="I598" s="4" t="inlineStr">
+        <is>
+          <t>NFLX's RSI is 11.3, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="599" ht="40" customHeight="1">
+      <c r="A599" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B599" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C599" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D599" s="8" t="inlineStr">
+        <is>
+          <t>PG</t>
+        </is>
+      </c>
+      <c r="E599" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F599" s="8" t="n">
+        <v>159.02</v>
+      </c>
+      <c r="G599" s="8" t="n">
+        <v>159.02</v>
+      </c>
+      <c r="H599" s="12" t="n">
+        <v>8.640000000000001</v>
+      </c>
+      <c r="I599" s="11" t="inlineStr">
+        <is>
+          <t>PG's 10-hour average ($160.27) dropped below its 30-hour average ($161.01). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="600" ht="40" customHeight="1">
+      <c r="A600" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B600" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C600" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D600" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E600" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F600" s="8" t="n">
+        <v>50.71</v>
+      </c>
+      <c r="G600" s="8" t="n">
+        <v>50.71</v>
+      </c>
+      <c r="H600" s="10" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="I600" s="11" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average ($50.81) dropped below its 30-hour average ($50.84). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="601" ht="40" customHeight="1">
+      <c r="A601" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B601" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C601" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D601" s="8" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E601" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F601" s="8" t="n">
+        <v>135.46</v>
+      </c>
+      <c r="G601" s="8" t="n">
+        <v>135.46</v>
+      </c>
+      <c r="H601" s="12" t="n">
+        <v>2.02</v>
+      </c>
+      <c r="I601" s="11" t="inlineStr">
+        <is>
+          <t>PEP's 10-hour average ($135.69) dropped below its 30-hour average ($135.86). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="602" ht="40" customHeight="1">
+      <c r="A602" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-26 18:57</t>
+        </is>
+      </c>
+      <c r="B602" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C602" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D602" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E602" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F602" s="8" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="G602" s="8" t="n">
+        <v>92.53</v>
+      </c>
+      <c r="H602" s="10" t="n">
+        <v>-2.3</v>
+      </c>
+      <c r="I602" s="11" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average ($92.60) dropped below its 30-hour average ($93.30). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -23269,19 +23538,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>635.9400000000001</v>
+        <v>629.38</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>465.42</v>
+        <v>309.74</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>35.94</v>
+        <v>29.38</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>5.99</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -23291,19 +23560,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>575.73</v>
+        <v>583.86</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>26.93</v>
+        <v>464.65</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-24.27</v>
+        <v>-16.14</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-4.04</v>
+        <v>-2.69</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -23343,7 +23612,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-23 22:54 UTC</t>
+          <t>Generated: 2026-10-26 18:57 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-27 18:29 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I602"/>
+  <dimension ref="A1:I605"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23451,6 +23451,119 @@
       <c r="I602" s="11" t="inlineStr">
         <is>
           <t>KO's 10-hour average ($92.60) dropped below its 30-hour average ($93.30). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="603" ht="40" customHeight="1">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 18:29</t>
+        </is>
+      </c>
+      <c r="B603" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C603" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="E603" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F603" s="2" t="n">
+        <v>141.75</v>
+      </c>
+      <c r="G603" s="2" t="n">
+        <v>141.75</v>
+      </c>
+      <c r="H603" s="2" t="inlineStr"/>
+      <c r="I603" s="4" t="inlineStr">
+        <is>
+          <t>MRK's RSI is 31.7, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="604" ht="40" customHeight="1">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-27 18:29</t>
+        </is>
+      </c>
+      <c r="B604" s="5" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C604" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E604" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F604" s="2" t="n">
+        <v>132.64</v>
+      </c>
+      <c r="G604" s="2" t="n">
+        <v>132.64</v>
+      </c>
+      <c r="H604" s="2" t="inlineStr"/>
+      <c r="I604" s="4" t="inlineStr">
+        <is>
+          <t>PEP's RSI is 27.4, which is below 35. RSI below 35 means the stock has been sold off heavily and is considered oversold — statistically likely to bounce back up.</t>
+        </is>
+      </c>
+    </row>
+    <row r="605" ht="40" customHeight="1">
+      <c r="A605" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-27 18:29</t>
+        </is>
+      </c>
+      <c r="B605" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C605" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D605" s="8" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E605" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F605" s="8" t="n">
+        <v>118.89</v>
+      </c>
+      <c r="G605" s="8" t="n">
+        <v>118.89</v>
+      </c>
+      <c r="H605" s="10" t="n">
+        <v>-0.32</v>
+      </c>
+      <c r="I605" s="11" t="inlineStr">
+        <is>
+          <t>WMT's 10-hour average ($119.56) dropped below its 30-hour average ($119.59). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
         </is>
       </c>
     </row>
@@ -23541,7 +23654,7 @@
         <v>629.38</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>309.74</v>
+        <v>35.34</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
@@ -23560,19 +23673,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>583.86</v>
+        <v>583.54</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>464.65</v>
+        <v>583.54</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-16.14</v>
+        <v>-16.46</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-2.69</v>
+        <v>-2.74</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -23612,7 +23725,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-26 23:35 UTC</t>
+          <t>Generated: 2026-10-27 18:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-28 18:34 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I605"/>
+  <dimension ref="A1:I606"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23564,6 +23564,43 @@
       <c r="I605" s="11" t="inlineStr">
         <is>
           <t>WMT's 10-hour average ($119.56) dropped below its 30-hour average ($119.59). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="606" ht="40" customHeight="1">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-28 18:34</t>
+        </is>
+      </c>
+      <c r="B606" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C606" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E606" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F606" s="2" t="n">
+        <v>50.84</v>
+      </c>
+      <c r="G606" s="2" t="n">
+        <v>101.68</v>
+      </c>
+      <c r="H606" s="2" t="inlineStr"/>
+      <c r="I606" s="4" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average price ($50.81) is above its 30-hour average ($50.80). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
         </is>
       </c>
     </row>
@@ -23676,7 +23713,7 @@
         <v>583.54</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>583.54</v>
+        <v>481.86</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
@@ -23725,7 +23762,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-27 23:30 UTC</t>
+          <t>Generated: 2026-10-28 18:34 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-29 18:44 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I606"/>
+  <dimension ref="A1:I609"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23601,6 +23601,121 @@
       <c r="I606" s="4" t="inlineStr">
         <is>
           <t>BAC's 10-hour average price ($50.81) is above its 30-hour average ($50.80). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="607" ht="40" customHeight="1">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:44</t>
+        </is>
+      </c>
+      <c r="B607" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C607" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>WMT</t>
+        </is>
+      </c>
+      <c r="E607" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F607" s="2" t="n">
+        <v>121.32</v>
+      </c>
+      <c r="G607" s="2" t="n">
+        <v>121.32</v>
+      </c>
+      <c r="H607" s="2" t="inlineStr"/>
+      <c r="I607" s="4" t="inlineStr">
+        <is>
+          <t>WMT is ranked #5 out of 25 stocks by momentum. It gained 2.20% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="608" ht="40" customHeight="1">
+      <c r="A608" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:44</t>
+        </is>
+      </c>
+      <c r="B608" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C608" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D608" s="8" t="inlineStr">
+        <is>
+          <t>MRK</t>
+        </is>
+      </c>
+      <c r="E608" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F608" s="8" t="n">
+        <v>146.31</v>
+      </c>
+      <c r="G608" s="8" t="n">
+        <v>146.31</v>
+      </c>
+      <c r="H608" s="12" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="I608" s="11" t="inlineStr">
+        <is>
+          <t>MRK's RSI climbed to 69.7, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="609" ht="40" customHeight="1">
+      <c r="A609" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-29 18:44</t>
+        </is>
+      </c>
+      <c r="B609" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C609" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D609" s="8" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E609" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F609" s="8" t="n">
+        <v>92.61</v>
+      </c>
+      <c r="G609" s="8" t="n">
+        <v>92.61</v>
+      </c>
+      <c r="H609" s="12" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I609" s="11" t="inlineStr">
+        <is>
+          <t>KO's RSI climbed to 66.8, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
         </is>
       </c>
     </row>
@@ -23669,7 +23784,7 @@
         <v>623.92</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>623.92</v>
+        <v>502.59</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -23688,19 +23803,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>629.38</v>
+        <v>634.01</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>35.34</v>
+        <v>274.26</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>29.38</v>
+        <v>34.01</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>4.9</v>
+        <v>5.67</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -23762,7 +23877,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-28 23:53 UTC</t>
+          <t>Generated: 2026-10-29 18:44 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
cycle 2026-10-30 18:20 UTC
</commit_message>
<xml_diff>
--- a/data/trades.xlsx
+++ b/data/trades.xlsx
@@ -564,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I609"/>
+  <dimension ref="A1:I617"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -23716,6 +23716,310 @@
       <c r="I609" s="11" t="inlineStr">
         <is>
           <t>KO's RSI climbed to 66.8, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="610" ht="40" customHeight="1">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B610" s="3" t="inlineStr">
+        <is>
+          <t>Momentum Agent</t>
+        </is>
+      </c>
+      <c r="C610" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E610" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F610" s="2" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="G610" s="2" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="H610" s="2" t="inlineStr"/>
+      <c r="I610" s="4" t="inlineStr">
+        <is>
+          <t>KO is ranked #5 out of 25 stocks by momentum. It gained 2.52% over the last 10 hours, showing strong upward price pressure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="611" ht="40" customHeight="1">
+      <c r="A611" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B611" s="13" t="inlineStr">
+        <is>
+          <t>RSI Agent</t>
+        </is>
+      </c>
+      <c r="C611" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D611" s="8" t="inlineStr">
+        <is>
+          <t>PEP</t>
+        </is>
+      </c>
+      <c r="E611" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F611" s="8" t="n">
+        <v>138.28</v>
+      </c>
+      <c r="G611" s="8" t="n">
+        <v>138.28</v>
+      </c>
+      <c r="H611" s="12" t="n">
+        <v>5.64</v>
+      </c>
+      <c r="I611" s="11" t="inlineStr">
+        <is>
+          <t>PEP's RSI climbed to 91.2, above 65. RSI above 65 means the stock is overbought — buyers are exhausted and a pullback is likely. Selling to lock in gains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="612" ht="40" customHeight="1">
+      <c r="A612" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B612" s="12" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C612" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D612" s="8" t="inlineStr">
+        <is>
+          <t>BAC</t>
+        </is>
+      </c>
+      <c r="E612" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="F612" s="8" t="n">
+        <v>49.87</v>
+      </c>
+      <c r="G612" s="8" t="n">
+        <v>99.73</v>
+      </c>
+      <c r="H612" s="10" t="n">
+        <v>-1.95</v>
+      </c>
+      <c r="I612" s="11" t="inlineStr">
+        <is>
+          <t>BAC's 10-hour average ($50.77) dropped below its 30-hour average ($50.84). This crossover is a classic bearish signal — the short-term trend has turned down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="613" ht="40" customHeight="1">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B613" s="6" t="inlineStr">
+        <is>
+          <t>MA Crossover</t>
+        </is>
+      </c>
+      <c r="C613" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>KO</t>
+        </is>
+      </c>
+      <c r="E613" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F613" s="2" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="G613" s="2" t="n">
+        <v>94.5</v>
+      </c>
+      <c r="H613" s="2" t="inlineStr"/>
+      <c r="I613" s="4" t="inlineStr">
+        <is>
+          <t>KO's 10-hour average price ($93.54) is above its 30-hour average ($92.53). This means short-term momentum is stronger than the longer trend — a bullish signal.</t>
+        </is>
+      </c>
+    </row>
+    <row r="614" ht="40" customHeight="1">
+      <c r="A614" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B614" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C614" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D614" s="8" t="inlineStr">
+        <is>
+          <t>DOW</t>
+        </is>
+      </c>
+      <c r="E614" s="8" t="n">
+        <v>6</v>
+      </c>
+      <c r="F614" s="8" t="n">
+        <v>34.57</v>
+      </c>
+      <c r="G614" s="8" t="n">
+        <v>207.42</v>
+      </c>
+      <c r="H614" s="12" t="n">
+        <v>29.07</v>
+      </c>
+      <c r="I614" s="11" t="inlineStr">
+        <is>
+          <t>TAKE-PROFIT: DOW is up 16.3% from the entry price (bought at $29.73, now $34.57). Locking in the gain before the price can reverse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="615" ht="40" customHeight="1">
+      <c r="A615" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B615" s="14" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C615" s="8" t="inlineStr">
+        <is>
+          <t>SELL</t>
+        </is>
+      </c>
+      <c r="D615" s="8" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="E615" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F615" s="8" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="G615" s="8" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="H615" s="12" t="n">
+        <v>11.93</v>
+      </c>
+      <c r="I615" s="11" t="inlineStr">
+        <is>
+          <t>TAKE-PROFIT: MO is up 17.9% from the entry price (bought at $66.58, now $78.51). Locking in the gain before the price can reverse.</t>
+        </is>
+      </c>
+    </row>
+    <row r="616" ht="40" customHeight="1">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B616" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C616" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>VZ</t>
+        </is>
+      </c>
+      <c r="E616" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="F616" s="2" t="n">
+        <v>45.06</v>
+      </c>
+      <c r="G616" s="2" t="n">
+        <v>135.19</v>
+      </c>
+      <c r="H616" s="2" t="inlineStr"/>
+      <c r="I616" s="4" t="inlineStr">
+        <is>
+          <t>VZ pays a 6.48% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($45.06) is above its 30-hour average ($43.81), confirming a healthy trend. Buying to collect steady income while holding.</t>
+        </is>
+      </c>
+    </row>
+    <row r="617" ht="40" customHeight="1">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-30 18:20</t>
+        </is>
+      </c>
+      <c r="B617" s="7" t="inlineStr">
+        <is>
+          <t>Dividend Agent</t>
+        </is>
+      </c>
+      <c r="C617" s="2" t="inlineStr">
+        <is>
+          <t>BUY</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>MO</t>
+        </is>
+      </c>
+      <c r="E617" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F617" s="2" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="G617" s="2" t="n">
+        <v>157.02</v>
+      </c>
+      <c r="H617" s="2" t="inlineStr"/>
+      <c r="I617" s="4" t="inlineStr">
+        <is>
+          <t>MO pays a 5.79% annual dividend yield, ranking it among the top dividend payers on the watchlist. Its price ($78.51) is above its 30-hour average ($74.77), confirming a healthy trend. Buying to collect steady income while holding.</t>
         </is>
       </c>
     </row>
@@ -23784,7 +24088,7 @@
         <v>623.92</v>
       </c>
       <c r="C2" s="16" t="n">
-        <v>502.59</v>
+        <v>408.1</v>
       </c>
       <c r="D2" s="16" t="n">
         <v>600</v>
@@ -23803,19 +24107,19 @@
         </is>
       </c>
       <c r="B3" s="16" t="n">
-        <v>634.01</v>
+        <v>639.65</v>
       </c>
       <c r="C3" s="16" t="n">
-        <v>274.26</v>
+        <v>412.54</v>
       </c>
       <c r="D3" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E3" s="17" t="n">
-        <v>34.01</v>
+        <v>39.65</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>5.67</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
@@ -23825,19 +24129,19 @@
         </is>
       </c>
       <c r="B4" s="16" t="n">
-        <v>583.54</v>
+        <v>581.59</v>
       </c>
       <c r="C4" s="16" t="n">
-        <v>481.86</v>
+        <v>487.1</v>
       </c>
       <c r="D4" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E4" s="19" t="n">
-        <v>-16.46</v>
+        <v>-18.41</v>
       </c>
       <c r="F4" s="19" t="n">
-        <v>-2.74</v>
+        <v>-3.07</v>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
@@ -23847,19 +24151,19 @@
         </is>
       </c>
       <c r="B5" s="16" t="n">
-        <v>526.6</v>
+        <v>567.6</v>
       </c>
       <c r="C5" s="16" t="n">
-        <v>25.43</v>
+        <v>19.14</v>
       </c>
       <c r="D5" s="16" t="n">
         <v>600</v>
       </c>
       <c r="E5" s="19" t="n">
-        <v>-73.40000000000001</v>
+        <v>-32.4</v>
       </c>
       <c r="F5" s="19" t="n">
-        <v>-12.23</v>
+        <v>-5.4</v>
       </c>
     </row>
     <row r="6">
@@ -23877,7 +24181,7 @@
     <row r="8">
       <c r="A8" s="21" t="inlineStr">
         <is>
-          <t>Generated: 2026-10-29 23:48 UTC</t>
+          <t>Generated: 2026-10-30 18:20 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>